<commit_message>
changes to data excel
</commit_message>
<xml_diff>
--- a/src/test/resources/testdata/data.xlsx
+++ b/src/test/resources/testdata/data.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="F:\SeleniumTraining\seleniumworkspace\com.orangehrm.automate\src\test\resources\testdata\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{6A21D7A7-6394-47E3-82D9-6911D196F9C2}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{3558E000-E865-4789-820A-BA93053194DB}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -26,7 +26,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="21" uniqueCount="11">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="17" uniqueCount="8">
   <si>
     <t>Admin</t>
   </si>
@@ -34,31 +34,22 @@
     <t>admin123</t>
   </si>
   <si>
-    <t>user_01</t>
-  </si>
-  <si>
-    <t>user_02</t>
-  </si>
-  <si>
     <t>Emily Jones</t>
   </si>
   <si>
-    <t>james123456</t>
-  </si>
-  <si>
     <t>ESS</t>
   </si>
   <si>
-    <t>Linda Anderson</t>
-  </si>
-  <si>
-    <t>linda1234567</t>
-  </si>
-  <si>
     <t>Ranga Akunuri</t>
   </si>
   <si>
-    <t>ranga1234567</t>
+    <t>linda12345678</t>
+  </si>
+  <si>
+    <t>ranga12345678</t>
+  </si>
+  <si>
+    <t>james1234568</t>
   </si>
 </sst>
 </file>
@@ -376,7 +367,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:B3"/>
+  <dimension ref="A1:B1"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="1" width="11" bestFit="1" customWidth="1"/>
@@ -389,22 +380,6 @@
       </c>
       <c r="B1" t="s">
         <v>1</v>
-      </c>
-    </row>
-    <row r="2" spans="1:2" x14ac:dyDescent="0.3">
-      <c r="A2" t="s">
-        <v>2</v>
-      </c>
-      <c r="B2" t="s">
-        <v>2</v>
-      </c>
-    </row>
-    <row r="3" spans="1:2" x14ac:dyDescent="0.3">
-      <c r="A3" t="s">
-        <v>3</v>
-      </c>
-      <c r="B3" t="s">
-        <v>3</v>
       </c>
     </row>
   </sheetData>
@@ -429,33 +404,33 @@
         <v>0</v>
       </c>
       <c r="B1" t="s">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="C1" t="s">
-        <v>5</v>
+        <v>7</v>
       </c>
       <c r="D1" t="s">
-        <v>5</v>
+        <v>7</v>
       </c>
       <c r="E1" t="s">
-        <v>5</v>
+        <v>7</v>
       </c>
     </row>
     <row r="2" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A2" t="s">
-        <v>6</v>
+        <v>3</v>
       </c>
       <c r="B2" t="s">
-        <v>7</v>
+        <v>2</v>
       </c>
       <c r="C2" t="s">
-        <v>8</v>
+        <v>5</v>
       </c>
       <c r="D2" t="s">
-        <v>8</v>
+        <v>5</v>
       </c>
       <c r="E2" t="s">
-        <v>8</v>
+        <v>5</v>
       </c>
     </row>
     <row r="3" spans="1:5" x14ac:dyDescent="0.3">
@@ -463,16 +438,16 @@
         <v>0</v>
       </c>
       <c r="B3" t="s">
-        <v>9</v>
+        <v>4</v>
       </c>
       <c r="C3" t="s">
-        <v>10</v>
+        <v>6</v>
       </c>
       <c r="D3" t="s">
-        <v>10</v>
+        <v>6</v>
       </c>
       <c r="E3" t="s">
-        <v>10</v>
+        <v>6</v>
       </c>
     </row>
   </sheetData>

</xml_diff>